<commit_message>
KRW: rename DV01 -> "KRD reformed", placed after KRD
Kevin wants the deliverable to be the delta table. Renamed the output sheet to
"KRD reformed" and positioned it immediately after KRD. It reads live off the KRD
delta row, so it reprices when notionals or the curve change.

Kevin confirmed the method for the sub-3M points: "just bump the points and see
what's the change in NPV." Verified that literally - added O/N/1W/1M/2M deposit
nodes to the curve and bumped each: the 10Y swap's NPV change is exactly 0.000000
for every one, 3M gives 1,718. So the zeros in the table are the genuine bump
result, not a skip. A 10Y swap has no sensitivity below 3M because its first
cashflow is at 3M and the 3M node is pinned by its own quote.

Table (placeholder notionals): buckets sum to -42,334,046 = the parallel DV01,
zero errors. Paste Kevin's real notionals into Amort-Set-up E20:E59 for the live
numbers.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/KRW_KevinGrid.xlsx
+++ b/bloomberg/KRW_KevinGrid.xlsx
@@ -7,12 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DV01" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quotes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interpolation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bootstrap" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Amort-Set-up" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KRD" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quotes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interpolation" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bootstrap" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Amort-Set-up" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KRD" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KRD reformed" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +26,7 @@
     <numFmt numFmtId="165" formatCode="0.00000000"/>
     <numFmt numFmtId="166" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -63,6 +63,12 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
       <color rgb="00808080"/>
       <sz val="9"/>
     </font>
@@ -116,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -138,6 +144,7 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -503,261 +510,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Delta - bump each tenor 1bp</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>KRW IRS loan hedge, 10Y. Each row = NPV change for +1bp on that tenor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Tenor</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>dv01</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>2D</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>1W</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>1M</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>2M</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>3M</t>
-        </is>
-      </c>
-      <c r="B9" s="5">
-        <f>KRD!S$69</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>6M</t>
-        </is>
-      </c>
-      <c r="B10" s="5">
-        <f>KRD!T$69</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>9M</t>
-        </is>
-      </c>
-      <c r="B11" s="5">
-        <f>KRD!U$69</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>1Y</t>
-        </is>
-      </c>
-      <c r="B12" s="5">
-        <f>KRD!V$69</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>2Y</t>
-        </is>
-      </c>
-      <c r="B13" s="5">
-        <f>KRD!W$69</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>3Y</t>
-        </is>
-      </c>
-      <c r="B14" s="5">
-        <f>KRD!X$69</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>4Y</t>
-        </is>
-      </c>
-      <c r="B15" s="5">
-        <f>KRD!Y$69</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>5Y</t>
-        </is>
-      </c>
-      <c r="B16" s="5">
-        <f>KRD!Z$69</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>7Y</t>
-        </is>
-      </c>
-      <c r="B17" s="5">
-        <f>KRD!AA$69</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>10Y</t>
-        </is>
-      </c>
-      <c r="B18" s="5">
-        <f>KRD!AB$69</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>12Y</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>15Y</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>20Y</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>25Y</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>30Y</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B24" s="7">
-        <f>SUM(B5:B23)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -969,7 +721,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2560,7 +2312,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5241,7 +4993,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6987,7 +6739,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12488,4 +12240,274 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Delta — 1bp per tenor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>KRW IRS loan hedge, 10Y. Each row = change in NPV for +1bp on that tenor. Live off the KRD delta row — reprices when the notionals or curve change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Tenor</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>dv01</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2D</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="21" t="inlineStr">
+        <is>
+          <t>2D–2M: no curve node below 3M / no swap sensitivity → 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>1W</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>12Y–30Y: past the 10Y maturity → 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="21" t="inlineStr">
+        <is>
+          <t>8Y/9Y risk sits in the 7Y and 10Y buckets (dropped as nodes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>2M</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>3M</t>
+        </is>
+      </c>
+      <c r="B9" s="5">
+        <f>KRD!S$69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>6M</t>
+        </is>
+      </c>
+      <c r="B10" s="5">
+        <f>KRD!T$69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>9M</t>
+        </is>
+      </c>
+      <c r="B11" s="5">
+        <f>KRD!U$69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>1Y</t>
+        </is>
+      </c>
+      <c r="B12" s="5">
+        <f>KRD!V$69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>2Y</t>
+        </is>
+      </c>
+      <c r="B13" s="5">
+        <f>KRD!W$69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>3Y</t>
+        </is>
+      </c>
+      <c r="B14" s="5">
+        <f>KRD!X$69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>4Y</t>
+        </is>
+      </c>
+      <c r="B15" s="5">
+        <f>KRD!Y$69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>5Y</t>
+        </is>
+      </c>
+      <c r="B16" s="5">
+        <f>KRD!Z$69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>7Y</t>
+        </is>
+      </c>
+      <c r="B17" s="5">
+        <f>KRD!AA$69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>10Y</t>
+        </is>
+      </c>
+      <c r="B18" s="5">
+        <f>KRD!AB$69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>12Y</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>15Y</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>20Y</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>25Y</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>30Y</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B24" s="7">
+        <f>SUM(B5:B23)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>